<commit_message>
+ Make Blue Slime enemy.
</commit_message>
<xml_diff>
--- a/Tool/data/GameNarrative.xlsx
+++ b/Tool/data/GameNarrative.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="8"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Actors" sheetId="1" r:id="rId1"/>
@@ -16,8 +16,7 @@
     <sheet name="QuestLines" sheetId="11" r:id="rId7"/>
     <sheet name="Quests" sheetId="12" r:id="rId8"/>
     <sheet name="Steps" sheetId="13" r:id="rId9"/>
-    <sheet name="Rewards" sheetId="10" r:id="rId10"/>
-    <sheet name="EventTemplate" sheetId="8" r:id="rId11"/>
+    <sheet name="EventTemplate" sheetId="8" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="166">
   <si>
     <t>ID</t>
   </si>
@@ -460,19 +459,7 @@
     <t>Mở thành tựa game</t>
   </si>
   <si>
-    <t>Count</t>
-  </si>
-  <si>
     <t>Default_01</t>
-  </si>
-  <si>
-    <t>Tofu_Soup</t>
-  </si>
-  <si>
-    <t>Jade</t>
-  </si>
-  <si>
-    <t>Coin</t>
   </si>
   <si>
     <t>QUEST_REWARD</t>
@@ -897,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>27</v>
@@ -1088,65 +1075,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C2" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C3" s="3">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>144</v>
-      </c>
-      <c r="B4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C4" s="3">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1302,13 +1230,13 @@
     </row>
     <row r="12" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -1357,7 +1285,7 @@
         <v>74</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C3" t="s">
         <v>16</v>
@@ -1368,7 +1296,7 @@
         <v>75</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -1379,7 +1307,7 @@
         <v>76</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C5" t="s">
         <v>16</v>
@@ -1387,10 +1315,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C6" t="s">
         <v>16</v>
@@ -1435,7 +1363,7 @@
         <v>62</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C2" t="s">
         <v>16</v>
@@ -1687,7 +1615,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>61</v>
@@ -1696,7 +1624,7 @@
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -1801,22 +1729,22 @@
         <v>57</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -1855,18 +1783,18 @@
         <v>101</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D2" s="3"/>
     </row>
@@ -1901,21 +1829,21 @@
         <v>101</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -1945,19 +1873,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>51</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>57</v>
@@ -1972,21 +1900,21 @@
         <v>139</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -1998,10 +1926,10 @@
         <v>1</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>144</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Remove Lines Component and add Nodes Component. Change manager Quest  Line
</commit_message>
<xml_diff>
--- a/Tool/data/GameNarrative.xlsx
+++ b/Tool/data/GameNarrative.xlsx
@@ -9,12 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Actors" sheetId="1" r:id="rId1"/>
     <sheet name="Dialogues" sheetId="2" r:id="rId2"/>
-    <sheet name="Lines" sheetId="3" r:id="rId3"/>
+    <sheet name="Nodes" sheetId="10" r:id="rId3"/>
     <sheet name="Choices" sheetId="4" r:id="rId4"/>
     <sheet name="QuestLines" sheetId="5" r:id="rId5"/>
     <sheet name="Quests" sheetId="6" r:id="rId6"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="211">
   <si>
     <t>ID</t>
   </si>
@@ -122,9 +122,6 @@
     <t>STR_DRAGON_KING_EATERN_SEA</t>
   </si>
   <si>
-    <t>Default_Dragon_king</t>
-  </si>
-  <si>
     <t>UI_EAST_SEA</t>
   </si>
   <si>
@@ -215,150 +212,18 @@
     <t>Default</t>
   </si>
   <si>
-    <t>Dragon_king_Choice_01</t>
-  </si>
-  <si>
     <t>Normal</t>
   </si>
   <si>
-    <t>Dragon_king_Choice_02</t>
-  </si>
-  <si>
-    <t>Dragon_king_Choice_03</t>
-  </si>
-  <si>
-    <t>Start_Quest_Dragon_king</t>
-  </si>
-  <si>
     <t>Start</t>
   </si>
   <si>
-    <t>DialogueID</t>
-  </si>
-  <si>
     <t>Text</t>
   </si>
   <si>
-    <t>HasChoice</t>
-  </si>
-  <si>
-    <t>L1-D1-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L1_D1_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L1-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L1_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L1-D3-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L1_D3_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L1_D4_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L2-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L2_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L3-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L3_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L4-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L4_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L5-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L5_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L6-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L6_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L7-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L7_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L8-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L8_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L9-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L9_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L10-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L10_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L11-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L11_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>L12-D2-Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L12_D2_Default_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>Default-Dragon_king</t>
-  </si>
-  <si>
-    <t>L_Deafult_Dragon_king_Eatern_Sea</t>
-  </si>
-  <si>
-    <t>LineID</t>
-  </si>
-  <si>
     <t>ActionChoiceType</t>
   </si>
   <si>
-    <t>NextDialogueID</t>
-  </si>
-  <si>
-    <t>Choice_01_Default_Wukong</t>
-  </si>
-  <si>
-    <t>Dia_Choice_01_Default_Wukong</t>
-  </si>
-  <si>
-    <t>DoNothing</t>
-  </si>
-  <si>
-    <t>Choice_03_Default_Wukong</t>
-  </si>
-  <si>
-    <t>Dia_Choice_03_Default_Wukong</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -371,12 +236,6 @@
     <t>Default_01</t>
   </si>
   <si>
-    <t>Default_QuestLine_Name</t>
-  </si>
-  <si>
-    <t>Default_QuestLine_Description</t>
-  </si>
-  <si>
     <t>Main</t>
   </si>
   <si>
@@ -389,12 +248,6 @@
     <t>EventID.1</t>
   </si>
   <si>
-    <t>Default_Quest_Name</t>
-  </si>
-  <si>
-    <t>Default_Quest_Description</t>
-  </si>
-  <si>
     <t>QUEST_REWARD</t>
   </si>
   <si>
@@ -645,13 +498,175 @@
   </si>
   <si>
     <t>Charracter</t>
+  </si>
+  <si>
+    <t>ActionType</t>
+  </si>
+  <si>
+    <t>NextNode</t>
+  </si>
+  <si>
+    <t>AcceptQuest</t>
+  </si>
+  <si>
+    <t>CompleteStep</t>
+  </si>
+  <si>
+    <t>GiveItem</t>
+  </si>
+  <si>
+    <t>OneShop</t>
+  </si>
+  <si>
+    <t>CloseDialogue</t>
+  </si>
+  <si>
+    <t>ContinueWithStep</t>
+  </si>
+  <si>
+    <t>WinningChoice</t>
+  </si>
+  <si>
+    <t>LosingChoice</t>
+  </si>
+  <si>
+    <t>IncompleteStep</t>
+  </si>
+  <si>
+    <t>DialogueType</t>
+  </si>
+  <si>
+    <t>Incompletion</t>
+  </si>
+  <si>
+    <t>NodeID</t>
+  </si>
+  <si>
+    <t>TargetNodeID</t>
+  </si>
+  <si>
+    <t>ChapterID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PrerequisiteQuestIDs </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RequiredLevel </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Name</t>
+  </si>
+  <si>
+    <t>QL_ChapterName</t>
+  </si>
+  <si>
+    <t>QL_ChapterName_Name</t>
+  </si>
+  <si>
+    <t>QL_ChapterName_Des</t>
+  </si>
+  <si>
+    <t>Q_ChapterName_QuestName</t>
+  </si>
+  <si>
+    <t>S_ChapterName_QuestName_01</t>
+  </si>
+  <si>
+    <t>Q_ChapterName_QuestName_Name</t>
+  </si>
+  <si>
+    <t>Q_ChapterName_QuestName_Des</t>
+  </si>
+  <si>
+    <t>DLG_ChapterName_QuestName_01_Start</t>
+  </si>
+  <si>
+    <t>DLG_ChapterName_QuestName_01_Incomplate</t>
+  </si>
+  <si>
+    <t>DLG_ChapterName_QuestName_01_Complate</t>
+  </si>
+  <si>
+    <t>DLG_Dragon_king_Eatern_Sea_Default</t>
+  </si>
+  <si>
+    <t>DLG_Dragon_king_Eatern_Sea_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>DLG_Dragon_king_Eatern_Sea_Default_Node_Ask</t>
+  </si>
+  <si>
+    <t>DLG_Dragon_king_Eatern_Sea_Default_Node_End</t>
+  </si>
+  <si>
+    <t>DLG_Dragon_king_Eatern_Sea_Default_Node_Answer</t>
+  </si>
+  <si>
+    <t>DLG_Dragon_king_Eatern_Sea_Default_Node_End_Dia</t>
+  </si>
+  <si>
+    <t>DLG_ChapterName_QuestName_01_Start_Node_Start</t>
+  </si>
+  <si>
+    <t>DLG_ChapterName_QuestName_01_Start_Node_Agree</t>
+  </si>
+  <si>
+    <t>DLG_ChapterName_QuestName_01_Start_Node_Refuse</t>
+  </si>
+  <si>
+    <t>STR_AGREE_QUEST</t>
+  </si>
+  <si>
+    <t>STR_REFUSE_QUEST</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Choice_Ask</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Choice_End</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Ask</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_End</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Answer</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_End_Dia</t>
+  </si>
+  <si>
+    <t>STR_DLG_ChapterName_QuestName_01_Start_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_ChapterName_QuestName_01_Start_Node_Agree</t>
+  </si>
+  <si>
+    <t>STR_DLG_ChapterName_QuestName_01_Start_Node_Refuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DialougeID </t>
+  </si>
+  <si>
+    <t>Completion</t>
+  </si>
+  <si>
+    <t>NextNodeID</t>
+  </si>
+  <si>
+    <t>node_end</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -665,8 +680,16 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -679,8 +702,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -703,11 +738,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -721,6 +767,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1028,7 +1082,7 @@
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -1144,101 +1198,101 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
+        <v>186</v>
+      </c>
+      <c r="D9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>32</v>
-      </c>
-      <c r="E9" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
         <v>34</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
         <v>35</v>
-      </c>
-      <c r="E10" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
         <v>37</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>38</v>
-      </c>
-      <c r="E11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
         <v>40</v>
       </c>
-      <c r="B12" t="s">
+      <c r="E12" t="s">
         <v>41</v>
-      </c>
-      <c r="E12" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" t="s">
         <v>43</v>
       </c>
-      <c r="B13" t="s">
+      <c r="E13" t="s">
         <v>44</v>
-      </c>
-      <c r="E13" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" t="s">
         <v>46</v>
       </c>
-      <c r="B14" t="s">
+      <c r="E14" t="s">
         <v>47</v>
-      </c>
-      <c r="E14" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
         <v>49</v>
       </c>
-      <c r="B15" t="s">
+      <c r="E15" t="s">
         <v>50</v>
-      </c>
-      <c r="E15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" t="s">
         <v>52</v>
       </c>
-      <c r="B16" t="s">
+      <c r="E16" t="s">
         <v>53</v>
-      </c>
-      <c r="E16" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" t="s">
         <v>55</v>
       </c>
-      <c r="B17" t="s">
+      <c r="E17" t="s">
         <v>56</v>
-      </c>
-      <c r="E17" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1248,81 +1302,102 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="31.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B2" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s">
-        <v>61</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B3" t="s">
         <v>62</v>
-      </c>
-      <c r="B3" t="s">
-        <v>63</v>
       </c>
       <c r="C3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>184</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>208</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" s="6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I11" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1332,369 +1407,292 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" customWidth="1"/>
+    <col min="4" max="4" width="54.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>70</v>
+      <c r="A1" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>71</v>
+      <c r="A2" s="6" t="s">
+        <v>187</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>186</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>73</v>
+      <c r="A3" s="6" t="s">
+        <v>188</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>186</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E3" t="b">
-        <v>0</v>
+        <v>200</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>75</v>
+      <c r="A4" s="6" t="s">
+        <v>189</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>186</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>77</v>
+      <c r="A5" s="6" t="s">
+        <v>190</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>186</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E5" t="b">
-        <v>0</v>
+        <v>202</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>78</v>
+      <c r="A6" s="6" t="s">
+        <v>191</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>186</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E6" t="b">
-        <v>0</v>
+        <v>203</v>
+      </c>
+      <c r="E6" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>192</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
         <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" t="b">
-        <v>0</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>193</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>183</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" t="b">
-        <v>0</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>194</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>183</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>85</v>
-      </c>
-      <c r="E9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" t="s">
-        <v>87</v>
-      </c>
-      <c r="E10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>90</v>
-      </c>
-      <c r="B12" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" t="s">
-        <v>91</v>
-      </c>
-      <c r="E12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>92</v>
-      </c>
-      <c r="B13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" t="s">
-        <v>95</v>
-      </c>
-      <c r="E14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" t="s">
-        <v>62</v>
-      </c>
-      <c r="C15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" t="s">
-        <v>97</v>
-      </c>
-      <c r="E15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" t="s">
-        <v>99</v>
-      </c>
-      <c r="E16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>100</v>
-      </c>
-      <c r="B17" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" t="s">
-        <v>101</v>
-      </c>
-      <c r="E17" t="b">
-        <v>0</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>102</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>187</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C2" t="s">
-        <v>106</v>
+        <v>197</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>158</v>
       </c>
       <c r="D2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>187</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" t="s">
-        <v>109</v>
+        <v>198</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>163</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E3" t="s">
-        <v>65</v>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" t="s">
+        <v>194</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I11" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I12" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I13" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I14" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I15" s="3" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1707,11 +1705,11 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1719,30 +1717,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>175</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>112</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>176</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>177</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D2" t="s">
-        <v>116</v>
+        <v>178</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1752,65 +1750,77 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.5703125" customWidth="1"/>
     <col min="6" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>118</v>
+        <v>71</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>176</v>
       </c>
       <c r="C2" t="s">
-        <v>120</v>
+        <v>181</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
+        <v>182</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="G2" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="H2" t="s">
-        <v>122</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1820,58 +1830,66 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" customWidth="1"/>
+    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="38.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>123</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>124</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>126</v>
+        <v>77</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>180</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>183</v>
       </c>
       <c r="G2" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1892,155 +1910,155 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>134</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>141</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
-        <v>142</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>143</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
-        <v>152</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s">
-        <v>156</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
-        <v>157</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>110</v>
       </c>
       <c r="D9" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>112</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>113</v>
       </c>
       <c r="D10" t="s">
-        <v>163</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="B11" t="s">
-        <v>165</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
-        <v>166</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>167</v>
+        <v>118</v>
       </c>
       <c r="D12" t="s">
-        <v>168</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2071,33 +2089,33 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>191</v>
+        <v>142</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>118</v>
+        <v>71</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>169</v>
+        <v>120</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>170</v>
+        <v>121</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>171</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>172</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>135</v>
       </c>
       <c r="C2" t="str">
         <f>B2&amp;"_DES"</f>
@@ -2108,16 +2126,16 @@
         <v>STR_DAILY_SLIME_TARGET</v>
       </c>
       <c r="E2" t="s">
-        <v>197</v>
+        <v>148</v>
       </c>
       <c r="F2" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>173</v>
+        <v>124</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>198</v>
+        <v>149</v>
       </c>
       <c r="I2">
         <v>3</v>
@@ -2125,10 +2143,10 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>125</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>134</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C9" si="1">B3&amp;"_DES"</f>
@@ -2142,13 +2160,13 @@
         <v>7</v>
       </c>
       <c r="F3" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>201</v>
+        <v>152</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>200</v>
+        <v>151</v>
       </c>
       <c r="I3">
         <v>3</v>
@@ -2156,10 +2174,10 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>179</v>
+        <v>130</v>
       </c>
       <c r="B4" t="s">
-        <v>185</v>
+        <v>136</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="1"/>
@@ -2170,13 +2188,13 @@
         <v>STR_DAILY_UPGADE_CHARACTER_TARGET</v>
       </c>
       <c r="E4" t="s">
-        <v>195</v>
+        <v>146</v>
       </c>
       <c r="F4" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>175</v>
+        <v>126</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4">
@@ -2185,10 +2203,10 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
+        <v>137</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="1"/>
@@ -2199,13 +2217,13 @@
         <v>STR_DAILY_UPGADE_WEAPON_TARGET</v>
       </c>
       <c r="E5" t="s">
-        <v>196</v>
+        <v>147</v>
       </c>
       <c r="F5" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5">
@@ -2214,10 +2232,10 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>178</v>
+        <v>129</v>
       </c>
       <c r="B6" t="s">
-        <v>187</v>
+        <v>138</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="1"/>
@@ -2228,13 +2246,13 @@
         <v>STR_DAILY_BATTLE_TARGET</v>
       </c>
       <c r="E6" t="s">
-        <v>194</v>
+        <v>145</v>
       </c>
       <c r="F6" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>202</v>
+        <v>153</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6">
@@ -2243,10 +2261,10 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>131</v>
       </c>
       <c r="B7" t="s">
-        <v>188</v>
+        <v>139</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="1"/>
@@ -2257,13 +2275,13 @@
         <v>STR_DAILY_SHOPPING_TARGET</v>
       </c>
       <c r="E7" t="s">
-        <v>192</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>203</v>
+        <v>154</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7">
@@ -2272,10 +2290,10 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>132</v>
       </c>
       <c r="B8" t="s">
-        <v>189</v>
+        <v>140</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="1"/>
@@ -2286,16 +2304,16 @@
         <v>STR_GACHA_CHARACTER_TARGET</v>
       </c>
       <c r="E8" t="s">
-        <v>193</v>
+        <v>144</v>
       </c>
       <c r="F8" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>204</v>
+        <v>155</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>205</v>
+        <v>156</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -2303,10 +2321,10 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>182</v>
+        <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>190</v>
+        <v>141</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="1"/>
@@ -2317,16 +2335,16 @@
         <v>STR_GACHA_WEAPON_TARGET</v>
       </c>
       <c r="E9" t="s">
-        <v>193</v>
+        <v>144</v>
       </c>
       <c r="F9" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>204</v>
+        <v>155</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>199</v>
+        <v>150</v>
       </c>
       <c r="I9">
         <v>1</v>

</xml_diff>

<commit_message>
+ Wormhole shader graph: Precision from Float to Half.
</commit_message>
<xml_diff>
--- a/Tool/data/GameNarrative.xlsx
+++ b/Tool/data/GameNarrative.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="641">
   <si>
     <t>ID</t>
   </si>
@@ -3168,6 +3168,9 @@
       <c r="D8" t="s">
         <v>203</v>
       </c>
+      <c r="E8" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
@@ -3181,6 +3184,9 @@
       </c>
       <c r="D9" t="s">
         <v>204</v>
+      </c>
+      <c r="E9" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>